<commit_message>
Improve cart system and category support
</commit_message>
<xml_diff>
--- a/Docs/03_Product_Master.xlsx
+++ b/Docs/03_Product_Master.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>Product ID</t>
   </si>
@@ -73,6 +73,39 @@
   </si>
   <si>
     <t>Sort Order</t>
+  </si>
+  <si>
+    <t>AAA0001</t>
+  </si>
+  <si>
+    <t>India Gate Basmati Rice</t>
+  </si>
+  <si>
+    <t>India Gate</t>
+  </si>
+  <si>
+    <t>AA</t>
+  </si>
+  <si>
+    <t>AAA</t>
+  </si>
+  <si>
+    <t>AAA0002</t>
+  </si>
+  <si>
+    <t>Daawat Basmati Rice</t>
+  </si>
+  <si>
+    <t>Daawat</t>
+  </si>
+  <si>
+    <t>AAA0003</t>
+  </si>
+  <si>
+    <t>Tilda Basmati Rice</t>
+  </si>
+  <si>
+    <t>Tilda</t>
   </si>
 </sst>
 </file>
@@ -113,9 +146,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,8 +454,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -475,6 +515,75 @@
       </c>
       <c r="R1" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2380</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4" s="2">
+        <v>980</v>
       </c>
     </row>
   </sheetData>

</xml_diff>